<commit_message>
LMDI: Merge pull request #73 from folkehelseinstituttet/fix/rename-festvirkestoff-slice
Endre slicenavn FestVirkestoff til FestLegemiddelVirkestoff 7f0ede665fb414cad3d1f5faafd3aae81ee9a6b0
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-medication.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-medication.xlsx
@@ -931,10 +931,10 @@
     <t>Medication.code.coding:Varenummer.userSelected</t>
   </si>
   <si>
-    <t>Medication.code.coding:FestVirkestoff</t>
-  </si>
-  <si>
-    <t>FestVirkestoff</t>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff</t>
+  </si>
+  <si>
+    <t>FestLegemiddelVirkestoff</t>
   </si>
   <si>
     <t>FEST-id for legemiddel virkestoff</t>
@@ -943,28 +943,28 @@
     <t>Unik identifikator (LegemiddelVirkestoff_ID) for rekvirering på virkestoffnivå i FEST.</t>
   </si>
   <si>
-    <t>Medication.code.coding:FestVirkestoff.id</t>
-  </si>
-  <si>
-    <t>Medication.code.coding:FestVirkestoff.extension</t>
-  </si>
-  <si>
-    <t>Medication.code.coding:FestVirkestoff.system</t>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.id</t>
+  </si>
+  <si>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.extension</t>
+  </si>
+  <si>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.system</t>
   </si>
   <si>
     <t>http://dmp.no/fhir/NamingSystem/festLegemiddelVirkestoff</t>
   </si>
   <si>
-    <t>Medication.code.coding:FestVirkestoff.version</t>
-  </si>
-  <si>
-    <t>Medication.code.coding:FestVirkestoff.code</t>
-  </si>
-  <si>
-    <t>Medication.code.coding:FestVirkestoff.display</t>
-  </si>
-  <si>
-    <t>Medication.code.coding:FestVirkestoff.userSelected</t>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.version</t>
+  </si>
+  <si>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.code</t>
+  </si>
+  <si>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.display</t>
+  </si>
+  <si>
+    <t>Medication.code.coding:FestLegemiddelVirkestoff.userSelected</t>
   </si>
   <si>
     <t>Medication.code.coding:LokaltLegemiddel</t>
@@ -1284,7 +1284,7 @@
     <t>Virkestoff(er) som inngår i legemiddelet. Skal fylles ut hvis code ikke har verdi. Bør fylles ut hvis code.coding[LokaltLegemiddel] har verdi.</t>
   </si>
   <si>
-    <t>For legemidler identifisert med FEST-koder (FestLegemiddeldose, FestLegemiddelMerkevare, FestLegemiddelpakning, FestVirkestoff, Varenummer) eller SNOMED CT er ingredient valgfritt, da virkestoffinformasjon kan hentes fra disse katalogene. For lokale legemidler anbefales det å oppgi ingredient for bedre sporbarhet.</t>
+    <t>For legemidler identifisert med FEST-koder (FestLegemiddeldose, FestLegemiddelMerkevare, FestLegemiddelpakning, FestLegemiddelVirkestoff, Varenummer) eller SNOMED CT er ingredient valgfritt, da virkestoffinformasjon kan hentes fra disse katalogene. For lokale legemidler anbefales det å oppgi ingredient for bedre sporbarhet.</t>
   </si>
   <si>
     <t>.scopesRole[typeCode=INGR]</t>

</xml_diff>

<commit_message>
LMDI: Merge pull request #75 from folkehelseinstituttet/fix/display-merkevare
Legg til display-beskrivelse for FestLegemiddelMerkevare ea8f5b0262dbe47ce56061a19b482ecec9b9b587
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-medication.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-medication.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4637" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4637" uniqueCount="459">
   <si>
     <t>Property</t>
   </si>
@@ -854,6 +854,9 @@
   </si>
   <si>
     <t>Medication.code.coding:FestLegemiddelMerkevare.display</t>
+  </si>
+  <si>
+    <t>Varenavn fra FEST</t>
   </si>
   <si>
     <t>Medication.code.coding:FestLegemiddelMerkevare.userSelected</t>
@@ -6183,7 +6186,7 @@
         <v>171</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="M39" t="s" s="2">
         <v>229</v>
@@ -6268,7 +6271,7 @@
     </row>
     <row r="40" hidden="true">
       <c r="A40" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B40" t="s" s="2">
         <v>235</v>
@@ -6384,13 +6387,13 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B41" t="s" s="2">
         <v>182</v>
       </c>
       <c r="C41" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D41" t="s" s="2">
         <v>77</v>
@@ -6415,10 +6418,10 @@
         <v>183</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="N41" t="s" s="2">
         <v>186</v>
@@ -6502,7 +6505,7 @@
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B42" t="s" s="2">
         <v>197</v>
@@ -6614,7 +6617,7 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B43" t="s" s="2">
         <v>199</v>
@@ -6728,7 +6731,7 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B44" t="s" s="2">
         <v>201</v>
@@ -6776,7 +6779,7 @@
         <v>77</v>
       </c>
       <c r="S44" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="T44" t="s" s="2">
         <v>77</v>
@@ -6844,7 +6847,7 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B45" t="s" s="2">
         <v>211</v>
@@ -6958,7 +6961,7 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B46" t="s" s="2">
         <v>219</v>
@@ -7072,7 +7075,7 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B47" t="s" s="2">
         <v>227</v>
@@ -7186,7 +7189,7 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B48" t="s" s="2">
         <v>235</v>
@@ -7302,13 +7305,13 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B49" t="s" s="2">
         <v>182</v>
       </c>
       <c r="C49" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D49" t="s" s="2">
         <v>77</v>
@@ -7333,10 +7336,10 @@
         <v>183</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N49" t="s" s="2">
         <v>186</v>
@@ -7420,7 +7423,7 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B50" t="s" s="2">
         <v>197</v>
@@ -7532,7 +7535,7 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B51" t="s" s="2">
         <v>199</v>
@@ -7646,7 +7649,7 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B52" t="s" s="2">
         <v>201</v>
@@ -7694,7 +7697,7 @@
         <v>77</v>
       </c>
       <c r="S52" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="T52" t="s" s="2">
         <v>77</v>
@@ -7762,7 +7765,7 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B53" t="s" s="2">
         <v>211</v>
@@ -7876,7 +7879,7 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B54" t="s" s="2">
         <v>219</v>
@@ -7905,7 +7908,7 @@
         <v>107</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M54" t="s" s="2">
         <v>221</v>
@@ -7990,7 +7993,7 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B55" t="s" s="2">
         <v>227</v>
@@ -8104,7 +8107,7 @@
     </row>
     <row r="56" hidden="true">
       <c r="A56" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B56" t="s" s="2">
         <v>235</v>
@@ -8220,13 +8223,13 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B57" t="s" s="2">
         <v>182</v>
       </c>
       <c r="C57" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D57" t="s" s="2">
         <v>77</v>
@@ -8251,10 +8254,10 @@
         <v>183</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="N57" t="s" s="2">
         <v>186</v>
@@ -8338,7 +8341,7 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B58" t="s" s="2">
         <v>197</v>
@@ -8450,7 +8453,7 @@
     </row>
     <row r="59" hidden="true">
       <c r="A59" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B59" t="s" s="2">
         <v>199</v>
@@ -8564,7 +8567,7 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B60" t="s" s="2">
         <v>201</v>
@@ -8612,7 +8615,7 @@
         <v>77</v>
       </c>
       <c r="S60" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="T60" t="s" s="2">
         <v>77</v>
@@ -8680,7 +8683,7 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B61" t="s" s="2">
         <v>211</v>
@@ -8794,7 +8797,7 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B62" t="s" s="2">
         <v>219</v>
@@ -8908,7 +8911,7 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B63" t="s" s="2">
         <v>227</v>
@@ -9022,7 +9025,7 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B64" t="s" s="2">
         <v>235</v>
@@ -9138,13 +9141,13 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B65" t="s" s="2">
         <v>182</v>
       </c>
       <c r="C65" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D65" t="s" s="2">
         <v>77</v>
@@ -9169,10 +9172,10 @@
         <v>183</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="N65" t="s" s="2">
         <v>186</v>
@@ -9256,7 +9259,7 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B66" t="s" s="2">
         <v>197</v>
@@ -9368,7 +9371,7 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B67" t="s" s="2">
         <v>199</v>
@@ -9482,7 +9485,7 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B68" t="s" s="2">
         <v>201</v>
@@ -9530,7 +9533,7 @@
         <v>77</v>
       </c>
       <c r="S68" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="T68" t="s" s="2">
         <v>77</v>
@@ -9598,7 +9601,7 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B69" t="s" s="2">
         <v>211</v>
@@ -9712,7 +9715,7 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B70" t="s" s="2">
         <v>219</v>
@@ -9741,7 +9744,7 @@
         <v>107</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="M70" t="s" s="2">
         <v>221</v>
@@ -9826,7 +9829,7 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B71" t="s" s="2">
         <v>227</v>
@@ -9855,7 +9858,7 @@
         <v>171</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="M71" t="s" s="2">
         <v>229</v>
@@ -9940,7 +9943,7 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B72" t="s" s="2">
         <v>235</v>
@@ -10056,13 +10059,13 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B73" t="s" s="2">
         <v>182</v>
       </c>
       <c r="C73" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D73" t="s" s="2">
         <v>77</v>
@@ -10087,10 +10090,10 @@
         <v>183</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="N73" t="s" s="2">
         <v>186</v>
@@ -10174,7 +10177,7 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B74" t="s" s="2">
         <v>197</v>
@@ -10286,7 +10289,7 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B75" t="s" s="2">
         <v>199</v>
@@ -10400,7 +10403,7 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B76" t="s" s="2">
         <v>201</v>
@@ -10448,7 +10451,7 @@
         <v>77</v>
       </c>
       <c r="S76" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="T76" t="s" s="2">
         <v>77</v>
@@ -10516,7 +10519,7 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B77" t="s" s="2">
         <v>211</v>
@@ -10630,7 +10633,7 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B78" t="s" s="2">
         <v>219</v>
@@ -10659,7 +10662,7 @@
         <v>107</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="M78" t="s" s="2">
         <v>221</v>
@@ -10744,7 +10747,7 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B79" t="s" s="2">
         <v>227</v>
@@ -10858,7 +10861,7 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B80" t="s" s="2">
         <v>235</v>
@@ -10974,10 +10977,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11003,16 +11006,16 @@
         <v>171</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="N81" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O81" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="P81" t="s" s="2">
         <v>77</v>
@@ -11061,7 +11064,7 @@
         <v>77</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>78</v>
@@ -11079,21 +11082,21 @@
         <v>77</v>
       </c>
       <c r="AL81" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM81" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN81" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11119,13 +11122,13 @@
         <v>107</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -11151,13 +11154,13 @@
         <v>77</v>
       </c>
       <c r="X82" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="Y82" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Z82" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="AA82" t="s" s="2">
         <v>77</v>
@@ -11175,7 +11178,7 @@
         <v>77</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>78</v>
@@ -11193,7 +11196,7 @@
         <v>77</v>
       </c>
       <c r="AL82" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AM82" t="s" s="2">
         <v>77</v>
@@ -11204,10 +11207,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11230,13 +11233,13 @@
         <v>88</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11287,7 +11290,7 @@
         <v>77</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
@@ -11302,24 +11305,24 @@
         <v>99</v>
       </c>
       <c r="AK83" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AM83" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AN83" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11345,13 +11348,13 @@
         <v>160</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -11377,13 +11380,13 @@
         <v>77</v>
       </c>
       <c r="X84" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="Y84" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="Z84" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>77</v>
@@ -11401,7 +11404,7 @@
         <v>77</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>78</v>
@@ -11416,24 +11419,24 @@
         <v>99</v>
       </c>
       <c r="AK84" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN84" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11542,10 +11545,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11656,10 +11659,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11685,13 +11688,13 @@
         <v>183</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="M87" t="s" s="2">
         <v>185</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="O87" t="s" s="2">
         <v>187</v>
@@ -11770,10 +11773,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -11882,10 +11885,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -11996,10 +11999,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12112,10 +12115,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12226,10 +12229,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12255,7 +12258,7 @@
         <v>107</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M92" t="s" s="2">
         <v>221</v>
@@ -12340,10 +12343,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12454,10 +12457,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12570,13 +12573,13 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C95" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D95" t="s" s="2">
         <v>77</v>
@@ -12601,7 +12604,7 @@
         <v>183</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="M95" t="s" s="2">
         <v>185</v>
@@ -12688,10 +12691,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12800,10 +12803,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -12914,10 +12917,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -12962,7 +12965,7 @@
         <v>77</v>
       </c>
       <c r="S98" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="T98" t="s" s="2">
         <v>77</v>
@@ -13030,10 +13033,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13144,10 +13147,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13173,7 +13176,7 @@
         <v>107</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="M100" t="s" s="2">
         <v>221</v>
@@ -13258,10 +13261,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -13287,7 +13290,7 @@
         <v>171</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="M101" t="s" s="2">
         <v>229</v>
@@ -13372,10 +13375,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13488,13 +13491,13 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C103" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D103" t="s" s="2">
         <v>77</v>
@@ -13519,7 +13522,7 @@
         <v>183</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="M103" t="s" s="2">
         <v>185</v>
@@ -13606,10 +13609,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -13718,10 +13721,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -13832,10 +13835,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -13880,7 +13883,7 @@
         <v>77</v>
       </c>
       <c r="S106" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="T106" t="s" s="2">
         <v>77</v>
@@ -13948,10 +13951,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14062,10 +14065,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14091,7 +14094,7 @@
         <v>107</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="M108" t="s" s="2">
         <v>221</v>
@@ -14176,10 +14179,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14290,10 +14293,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14406,10 +14409,10 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14435,16 +14438,16 @@
         <v>171</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="O111" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="P111" t="s" s="2">
         <v>77</v>
@@ -14493,7 +14496,7 @@
         <v>77</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
@@ -14511,21 +14514,21 @@
         <v>77</v>
       </c>
       <c r="AL111" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM111" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -14548,13 +14551,13 @@
         <v>88</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
@@ -14605,7 +14608,7 @@
         <v>77</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>78</v>
@@ -14623,7 +14626,7 @@
         <v>77</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AM112" t="s" s="2">
         <v>77</v>
@@ -14634,10 +14637,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -14660,16 +14663,16 @@
         <v>77</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="O113" s="2"/>
       <c r="P113" t="s" s="2">
@@ -14719,7 +14722,7 @@
         <v>77</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
@@ -14737,7 +14740,7 @@
         <v>77</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="AM113" t="s" s="2">
         <v>77</v>
@@ -14748,10 +14751,10 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -14860,10 +14863,10 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -14974,14 +14977,14 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E116" s="2"/>
       <c r="F116" t="s" s="2">
@@ -15003,10 +15006,10 @@
         <v>132</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="N116" t="s" s="2">
         <v>149</v>
@@ -15061,7 +15064,7 @@
         <v>77</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>78</v>
@@ -15090,10 +15093,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15116,17 +15119,17 @@
         <v>77</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="P117" t="s" s="2">
         <v>77</v>
@@ -15163,7 +15166,7 @@
         <v>77</v>
       </c>
       <c r="AB117" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="AC117" s="2"/>
       <c r="AD117" t="s" s="2">
@@ -15173,7 +15176,7 @@
         <v>136</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>87</v>
@@ -15191,24 +15194,24 @@
         <v>166</v>
       </c>
       <c r="AL117" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="AM117" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN117" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C118" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D118" t="s" s="2">
         <v>77</v>
@@ -15230,17 +15233,17 @@
         <v>77</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="P118" t="s" s="2">
         <v>77</v>
@@ -15289,7 +15292,7 @@
         <v>77</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>87</v>
@@ -15307,24 +15310,24 @@
         <v>166</v>
       </c>
       <c r="AL118" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="AM118" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN118" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C119" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D119" t="s" s="2">
         <v>77</v>
@@ -15349,14 +15352,14 @@
         <v>160</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="P119" t="s" s="2">
         <v>77</v>
@@ -15403,7 +15406,7 @@
         <v>77</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>87</v>
@@ -15421,21 +15424,21 @@
         <v>166</v>
       </c>
       <c r="AL119" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="AM119" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN119" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -15461,14 +15464,14 @@
         <v>236</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="P120" t="s" s="2">
         <v>77</v>
@@ -15517,7 +15520,7 @@
         <v>77</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>78</v>
@@ -15535,7 +15538,7 @@
         <v>77</v>
       </c>
       <c r="AL120" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="AM120" t="s" s="2">
         <v>77</v>
@@ -15546,10 +15549,10 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -15572,13 +15575,13 @@
         <v>77</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="L121" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -15629,7 +15632,7 @@
         <v>77</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>78</v>
@@ -15644,24 +15647,24 @@
         <v>99</v>
       </c>
       <c r="AK121" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="AL121" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="AM121" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN121" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -15684,13 +15687,13 @@
         <v>77</v>
       </c>
       <c r="K122" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
@@ -15741,7 +15744,7 @@
         <v>77</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>78</v>
@@ -15756,10 +15759,10 @@
         <v>99</v>
       </c>
       <c r="AK122" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AL122" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="AM122" t="s" s="2">
         <v>77</v>
@@ -15770,10 +15773,10 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -15882,10 +15885,10 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -15996,14 +15999,14 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E125" s="2"/>
       <c r="F125" t="s" s="2">
@@ -16025,10 +16028,10 @@
         <v>132</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="N125" t="s" s="2">
         <v>149</v>
@@ -16083,7 +16086,7 @@
         <v>77</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>78</v>
@@ -16112,10 +16115,10 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16141,10 +16144,10 @@
         <v>171</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -16195,7 +16198,7 @@
         <v>77</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>78</v>
@@ -16210,7 +16213,7 @@
         <v>99</v>
       </c>
       <c r="AK126" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AL126" t="s" s="2">
         <v>157</v>
@@ -16219,15 +16222,15 @@
         <v>77</v>
       </c>
       <c r="AN126" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -16250,13 +16253,13 @@
         <v>77</v>
       </c>
       <c r="K127" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L127" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M127" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
@@ -16307,7 +16310,7 @@
         <v>77</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>78</v>
@@ -16322,16 +16325,16 @@
         <v>99</v>
       </c>
       <c r="AK127" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AL127" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="AM127" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN127" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LMDI: Oppdater display ^short for FEST-kodesystem i Legemiddel-profil
Lukker #68 b109e838aad9a6d066fedddc75bfe58bd269b909
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-medication.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-medication.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4637" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4637" uniqueCount="460">
   <si>
     <t>Property</t>
   </si>
@@ -735,7 +735,7 @@
     <t>Medication.code.coding.display</t>
   </si>
   <si>
-    <t>Representation defined by the system</t>
+    <t>NavnFormStyrke fra FEST</t>
   </si>
   <si>
     <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
@@ -856,7 +856,7 @@
     <t>Medication.code.coding:FestLegemiddelMerkevare.display</t>
   </si>
   <si>
-    <t>Varenavn fra FEST</t>
+    <t>Varenavn eller NavnFormStyrke fra FEST</t>
   </si>
   <si>
     <t>Medication.code.coding:FestLegemiddelMerkevare.userSelected</t>
@@ -1046,6 +1046,9 @@
   </si>
   <si>
     <t>Medication.code.coding:SCT.display</t>
+  </si>
+  <si>
+    <t>Representation defined by the system</t>
   </si>
   <si>
     <t>Medication.code.coding:SCT.userSelected</t>
@@ -7104,7 +7107,7 @@
         <v>171</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="M47" t="s" s="2">
         <v>229</v>
@@ -8022,7 +8025,7 @@
         <v>171</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>228</v>
+        <v>268</v>
       </c>
       <c r="M55" t="s" s="2">
         <v>229</v>
@@ -10776,7 +10779,7 @@
         <v>171</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>228</v>
+        <v>332</v>
       </c>
       <c r="M79" t="s" s="2">
         <v>229</v>
@@ -10861,7 +10864,7 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B80" t="s" s="2">
         <v>235</v>
@@ -10977,10 +10980,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11006,16 +11009,16 @@
         <v>171</v>
       </c>
       <c r="L81" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M81" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N81" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="O81" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P81" t="s" s="2">
         <v>77</v>
@@ -11064,7 +11067,7 @@
         <v>77</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>78</v>
@@ -11082,21 +11085,21 @@
         <v>77</v>
       </c>
       <c r="AL81" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AM81" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN81" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11122,13 +11125,13 @@
         <v>107</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="N82" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="O82" s="2"/>
       <c r="P82" t="s" s="2">
@@ -11154,13 +11157,13 @@
         <v>77</v>
       </c>
       <c r="X82" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="Y82" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="Z82" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AA82" t="s" s="2">
         <v>77</v>
@@ -11178,7 +11181,7 @@
         <v>77</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>78</v>
@@ -11196,7 +11199,7 @@
         <v>77</v>
       </c>
       <c r="AL82" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AM82" t="s" s="2">
         <v>77</v>
@@ -11207,10 +11210,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11233,13 +11236,13 @@
         <v>88</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11290,7 +11293,7 @@
         <v>77</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
@@ -11305,24 +11308,24 @@
         <v>99</v>
       </c>
       <c r="AK83" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="AM83" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="AN83" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11348,13 +11351,13 @@
         <v>160</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="N84" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="O84" s="2"/>
       <c r="P84" t="s" s="2">
@@ -11380,13 +11383,13 @@
         <v>77</v>
       </c>
       <c r="X84" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="Y84" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Z84" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>77</v>
@@ -11404,7 +11407,7 @@
         <v>77</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>78</v>
@@ -11419,24 +11422,24 @@
         <v>99</v>
       </c>
       <c r="AK84" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN84" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11545,10 +11548,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11659,10 +11662,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11688,13 +11691,13 @@
         <v>183</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="M87" t="s" s="2">
         <v>185</v>
       </c>
       <c r="N87" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="O87" t="s" s="2">
         <v>187</v>
@@ -11773,10 +11776,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -11885,10 +11888,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -11999,10 +12002,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12115,10 +12118,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12229,10 +12232,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12258,7 +12261,7 @@
         <v>107</v>
       </c>
       <c r="L92" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M92" t="s" s="2">
         <v>221</v>
@@ -12343,10 +12346,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12372,7 +12375,7 @@
         <v>171</v>
       </c>
       <c r="L93" t="s" s="2">
-        <v>228</v>
+        <v>332</v>
       </c>
       <c r="M93" t="s" s="2">
         <v>229</v>
@@ -12457,10 +12460,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12573,13 +12576,13 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C95" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D95" t="s" s="2">
         <v>77</v>
@@ -12604,7 +12607,7 @@
         <v>183</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="M95" t="s" s="2">
         <v>185</v>
@@ -12691,10 +12694,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12803,10 +12806,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -12917,10 +12920,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -12965,7 +12968,7 @@
         <v>77</v>
       </c>
       <c r="S98" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="T98" t="s" s="2">
         <v>77</v>
@@ -13033,10 +13036,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13147,10 +13150,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13176,7 +13179,7 @@
         <v>107</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="M100" t="s" s="2">
         <v>221</v>
@@ -13261,10 +13264,10 @@
     </row>
     <row r="101">
       <c r="A101" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -13290,7 +13293,7 @@
         <v>171</v>
       </c>
       <c r="L101" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="M101" t="s" s="2">
         <v>229</v>
@@ -13375,10 +13378,10 @@
     </row>
     <row r="102" hidden="true">
       <c r="A102" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B102" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C102" s="2"/>
       <c r="D102" t="s" s="2">
@@ -13491,10 +13494,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C103" t="s" s="2">
         <v>321</v>
@@ -13522,7 +13525,7 @@
         <v>183</v>
       </c>
       <c r="L103" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="M103" t="s" s="2">
         <v>185</v>
@@ -13609,10 +13612,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -13721,10 +13724,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -13835,10 +13838,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -13951,10 +13954,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -14065,10 +14068,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -14094,7 +14097,7 @@
         <v>107</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="M108" t="s" s="2">
         <v>221</v>
@@ -14179,10 +14182,10 @@
     </row>
     <row r="109">
       <c r="A109" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -14208,7 +14211,7 @@
         <v>171</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>228</v>
+        <v>332</v>
       </c>
       <c r="M109" t="s" s="2">
         <v>229</v>
@@ -14293,10 +14296,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -14409,10 +14412,10 @@
     </row>
     <row r="111" hidden="true">
       <c r="A111" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B111" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C111" s="2"/>
       <c r="D111" t="s" s="2">
@@ -14438,16 +14441,16 @@
         <v>171</v>
       </c>
       <c r="L111" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M111" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="N111" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="O111" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P111" t="s" s="2">
         <v>77</v>
@@ -14496,7 +14499,7 @@
         <v>77</v>
       </c>
       <c r="AF111" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AG111" t="s" s="2">
         <v>78</v>
@@ -14514,21 +14517,21 @@
         <v>77</v>
       </c>
       <c r="AL111" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AM111" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN111" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="112" hidden="true">
       <c r="A112" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B112" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C112" s="2"/>
       <c r="D112" t="s" s="2">
@@ -14551,13 +14554,13 @@
         <v>88</v>
       </c>
       <c r="K112" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="L112" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="M112" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="N112" s="2"/>
       <c r="O112" s="2"/>
@@ -14608,7 +14611,7 @@
         <v>77</v>
       </c>
       <c r="AF112" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="AG112" t="s" s="2">
         <v>78</v>
@@ -14626,7 +14629,7 @@
         <v>77</v>
       </c>
       <c r="AL112" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AM112" t="s" s="2">
         <v>77</v>
@@ -14637,10 +14640,10 @@
     </row>
     <row r="113" hidden="true">
       <c r="A113" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B113" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C113" s="2"/>
       <c r="D113" t="s" s="2">
@@ -14663,16 +14666,16 @@
         <v>77</v>
       </c>
       <c r="K113" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="L113" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M113" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="N113" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="O113" s="2"/>
       <c r="P113" t="s" s="2">
@@ -14722,7 +14725,7 @@
         <v>77</v>
       </c>
       <c r="AF113" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="AG113" t="s" s="2">
         <v>78</v>
@@ -14740,7 +14743,7 @@
         <v>77</v>
       </c>
       <c r="AL113" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="AM113" t="s" s="2">
         <v>77</v>
@@ -14751,10 +14754,10 @@
     </row>
     <row r="114" hidden="true">
       <c r="A114" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B114" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C114" s="2"/>
       <c r="D114" t="s" s="2">
@@ -14863,10 +14866,10 @@
     </row>
     <row r="115" hidden="true">
       <c r="A115" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B115" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C115" s="2"/>
       <c r="D115" t="s" s="2">
@@ -14977,14 +14980,14 @@
     </row>
     <row r="116" hidden="true">
       <c r="A116" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B116" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C116" s="2"/>
       <c r="D116" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E116" s="2"/>
       <c r="F116" t="s" s="2">
@@ -15006,10 +15009,10 @@
         <v>132</v>
       </c>
       <c r="L116" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M116" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N116" t="s" s="2">
         <v>149</v>
@@ -15064,7 +15067,7 @@
         <v>77</v>
       </c>
       <c r="AF116" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AG116" t="s" s="2">
         <v>78</v>
@@ -15093,10 +15096,10 @@
     </row>
     <row r="117" hidden="true">
       <c r="A117" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B117" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C117" s="2"/>
       <c r="D117" t="s" s="2">
@@ -15119,17 +15122,17 @@
         <v>77</v>
       </c>
       <c r="K117" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="L117" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="M117" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="N117" s="2"/>
       <c r="O117" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="P117" t="s" s="2">
         <v>77</v>
@@ -15166,7 +15169,7 @@
         <v>77</v>
       </c>
       <c r="AB117" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="AC117" s="2"/>
       <c r="AD117" t="s" s="2">
@@ -15176,7 +15179,7 @@
         <v>136</v>
       </c>
       <c r="AF117" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AG117" t="s" s="2">
         <v>87</v>
@@ -15194,24 +15197,24 @@
         <v>166</v>
       </c>
       <c r="AL117" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AM117" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN117" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="118" hidden="true">
       <c r="A118" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B118" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C118" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D118" t="s" s="2">
         <v>77</v>
@@ -15233,17 +15236,17 @@
         <v>77</v>
       </c>
       <c r="K118" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="L118" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="M118" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="N118" s="2"/>
       <c r="O118" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="P118" t="s" s="2">
         <v>77</v>
@@ -15292,7 +15295,7 @@
         <v>77</v>
       </c>
       <c r="AF118" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AG118" t="s" s="2">
         <v>87</v>
@@ -15310,24 +15313,24 @@
         <v>166</v>
       </c>
       <c r="AL118" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AM118" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN118" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="119" hidden="true">
       <c r="A119" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="B119" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C119" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D119" t="s" s="2">
         <v>77</v>
@@ -15352,14 +15355,14 @@
         <v>160</v>
       </c>
       <c r="L119" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="M119" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="N119" s="2"/>
       <c r="O119" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="P119" t="s" s="2">
         <v>77</v>
@@ -15406,7 +15409,7 @@
         <v>77</v>
       </c>
       <c r="AF119" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="AG119" t="s" s="2">
         <v>87</v>
@@ -15424,21 +15427,21 @@
         <v>166</v>
       </c>
       <c r="AL119" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="AM119" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN119" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="120" hidden="true">
       <c r="A120" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B120" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C120" s="2"/>
       <c r="D120" t="s" s="2">
@@ -15464,14 +15467,14 @@
         <v>236</v>
       </c>
       <c r="L120" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M120" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="N120" s="2"/>
       <c r="O120" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="P120" t="s" s="2">
         <v>77</v>
@@ -15520,7 +15523,7 @@
         <v>77</v>
       </c>
       <c r="AF120" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="AG120" t="s" s="2">
         <v>78</v>
@@ -15538,7 +15541,7 @@
         <v>77</v>
       </c>
       <c r="AL120" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="AM120" t="s" s="2">
         <v>77</v>
@@ -15549,10 +15552,10 @@
     </row>
     <row r="121" hidden="true">
       <c r="A121" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C121" s="2"/>
       <c r="D121" t="s" s="2">
@@ -15575,13 +15578,13 @@
         <v>77</v>
       </c>
       <c r="K121" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="L121" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -15632,7 +15635,7 @@
         <v>77</v>
       </c>
       <c r="AF121" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="AG121" t="s" s="2">
         <v>78</v>
@@ -15647,24 +15650,24 @@
         <v>99</v>
       </c>
       <c r="AK121" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="AL121" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="AM121" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN121" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -15687,13 +15690,13 @@
         <v>77</v>
       </c>
       <c r="K122" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
@@ -15744,7 +15747,7 @@
         <v>77</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>78</v>
@@ -15759,10 +15762,10 @@
         <v>99</v>
       </c>
       <c r="AK122" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AL122" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="AM122" t="s" s="2">
         <v>77</v>
@@ -15773,10 +15776,10 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
@@ -15885,10 +15888,10 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C124" s="2"/>
       <c r="D124" t="s" s="2">
@@ -15999,14 +16002,14 @@
     </row>
     <row r="125" hidden="true">
       <c r="A125" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E125" s="2"/>
       <c r="F125" t="s" s="2">
@@ -16028,10 +16031,10 @@
         <v>132</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="N125" t="s" s="2">
         <v>149</v>
@@ -16086,7 +16089,7 @@
         <v>77</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>78</v>
@@ -16115,10 +16118,10 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16144,10 +16147,10 @@
         <v>171</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -16198,7 +16201,7 @@
         <v>77</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>78</v>
@@ -16213,7 +16216,7 @@
         <v>99</v>
       </c>
       <c r="AK126" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AL126" t="s" s="2">
         <v>157</v>
@@ -16222,15 +16225,15 @@
         <v>77</v>
       </c>
       <c r="AN126" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="127" hidden="true">
       <c r="A127" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -16253,13 +16256,13 @@
         <v>77</v>
       </c>
       <c r="K127" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="L127" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="M127" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
@@ -16310,7 +16313,7 @@
         <v>77</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>78</v>
@@ -16325,16 +16328,16 @@
         <v>99</v>
       </c>
       <c r="AK127" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AL127" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="AM127" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN127" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LMDI: Merge pull request #104 from folkehelseinstituttet/roar/automatisk-currentbuild-publisering
Publiser currentbuild automatisk ved push til main ad8dde0c71354bd04ce34fd687fc57c5dc72285f
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-medication.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-medication.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$132</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4637" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4814" uniqueCount="478">
   <si>
     <t>Property</t>
   </si>
@@ -1383,16 +1383,69 @@
     <t>Medication.ingredient.strength</t>
   </si>
   <si>
-    <t>Quantity of ingredient present</t>
-  </si>
-  <si>
-    <t>Specifies how many (or how much) of the items there are in this Medication.  For example, 250 mg per tablet.  This is expressed as a ratio where the numerator is 250mg and the denominator is 1 tablet.</t>
+    <t>Styrken av ingrediensen i det rekvirerte/administrerte legemidlet.</t>
   </si>
   <si>
     <t>//element(*,DrugCodedType)/Strength</t>
   </si>
   <si>
     <t>RXC-3-Component Amount &amp; RXC-4-Component Units  if medication: RXO-2-Requested Give Amount - Minimum &amp; RXO-4-Requested Give Units / RXO-3-Requested Give Amount - Maximum &amp; RXO-4-Requested Give Units / RXO-11-Requested Dispense Amount &amp; RXO-12-Requested Dispense Units / RXE-3-Give Amount - Minimum &amp; RXE-5-Give Units / RXE-4-Give Amount - Maximum &amp; RXE-5-Give Units / RXE-10-Dispense Amount &amp; RXE-10-Dispense Units</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.strength.id</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.strength.extension</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.strength.extension:mengde</t>
+  </si>
+  <si>
+    <t>mengde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.no/fhir/ig/lmdi/StructureDefinition/lmdi-ingredient-strength}
+</t>
+  </si>
+  <si>
+    <t>Mengde ingrediens i det rekvirerte/administrerte legemidlet.</t>
+  </si>
+  <si>
+    <t>Mengde ingrediens i det rekvirerte/administrerte legemidlet, angitt som volum eller mengde virkestoff (Quantity), eller som kode (qs, trace). Brukes i stedet for teller og nevner i strength.</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.strength.numerator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantity
+</t>
+  </si>
+  <si>
+    <t>Numerator value</t>
+  </si>
+  <si>
+    <t>The value of the numerator.</t>
+  </si>
+  <si>
+    <t>Ratio.numerator</t>
+  </si>
+  <si>
+    <t>.numerator</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.strength.denominator</t>
+  </si>
+  <si>
+    <t>Denominator value</t>
+  </si>
+  <si>
+    <t>The value of the denominator.</t>
+  </si>
+  <si>
+    <t>Ratio.denominator</t>
+  </si>
+  <si>
+    <t>.denominator</t>
   </si>
   <si>
     <t>Medication.batch</t>
@@ -1769,11 +1822,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN127"/>
+  <dimension ref="A1:AN132"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="51.640625" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="32.79296875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="35.77734375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.73046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -15587,7 +15640,7 @@
         <v>440</v>
       </c>
       <c r="M121" t="s" s="2">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="N121" s="2"/>
       <c r="O121" s="2"/>
@@ -15653,7 +15706,7 @@
         <v>99</v>
       </c>
       <c r="AK121" t="s" s="2">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="AL121" t="s" s="2">
         <v>408</v>
@@ -15662,15 +15715,15 @@
         <v>77</v>
       </c>
       <c r="AN121" t="s" s="2">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="122" hidden="true">
+      <c r="A122" t="s" s="2">
         <v>443</v>
       </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="s" s="2">
-        <v>444</v>
-      </c>
       <c r="B122" t="s" s="2">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C122" s="2"/>
       <c r="D122" t="s" s="2">
@@ -15684,7 +15737,7 @@
         <v>87</v>
       </c>
       <c r="H122" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I122" t="s" s="2">
         <v>77</v>
@@ -15693,13 +15746,13 @@
         <v>77</v>
       </c>
       <c r="K122" t="s" s="2">
-        <v>410</v>
+        <v>172</v>
       </c>
       <c r="L122" t="s" s="2">
-        <v>445</v>
+        <v>173</v>
       </c>
       <c r="M122" t="s" s="2">
-        <v>446</v>
+        <v>174</v>
       </c>
       <c r="N122" s="2"/>
       <c r="O122" s="2"/>
@@ -15750,7 +15803,7 @@
         <v>77</v>
       </c>
       <c r="AF122" t="s" s="2">
-        <v>444</v>
+        <v>175</v>
       </c>
       <c r="AG122" t="s" s="2">
         <v>78</v>
@@ -15762,13 +15815,13 @@
         <v>77</v>
       </c>
       <c r="AJ122" t="s" s="2">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="AK122" t="s" s="2">
-        <v>355</v>
+        <v>77</v>
       </c>
       <c r="AL122" t="s" s="2">
-        <v>447</v>
+        <v>176</v>
       </c>
       <c r="AM122" t="s" s="2">
         <v>77</v>
@@ -15779,21 +15832,21 @@
     </row>
     <row r="123" hidden="true">
       <c r="A123" t="s" s="2">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="C123" s="2"/>
       <c r="D123" t="s" s="2">
-        <v>77</v>
+        <v>147</v>
       </c>
       <c r="E123" s="2"/>
       <c r="F123" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G123" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H123" t="s" s="2">
         <v>77</v>
@@ -15805,15 +15858,17 @@
         <v>77</v>
       </c>
       <c r="K123" t="s" s="2">
-        <v>172</v>
+        <v>132</v>
       </c>
       <c r="L123" t="s" s="2">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="M123" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N123" s="2"/>
+        <v>179</v>
+      </c>
+      <c r="N123" t="s" s="2">
+        <v>150</v>
+      </c>
       <c r="O123" s="2"/>
       <c r="P123" t="s" s="2">
         <v>77</v>
@@ -15850,31 +15905,31 @@
         <v>77</v>
       </c>
       <c r="AB123" t="s" s="2">
-        <v>77</v>
+        <v>135</v>
       </c>
       <c r="AC123" t="s" s="2">
-        <v>77</v>
+        <v>180</v>
       </c>
       <c r="AD123" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE123" t="s" s="2">
-        <v>77</v>
+        <v>181</v>
       </c>
       <c r="AF123" t="s" s="2">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="AG123" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH123" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI123" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ123" t="s" s="2">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="AK123" t="s" s="2">
         <v>77</v>
@@ -15891,21 +15946,23 @@
     </row>
     <row r="124" hidden="true">
       <c r="A124" t="s" s="2">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="C124" s="2"/>
+        <v>444</v>
+      </c>
+      <c r="C124" t="s" s="2">
+        <v>446</v>
+      </c>
       <c r="D124" t="s" s="2">
-        <v>147</v>
+        <v>77</v>
       </c>
       <c r="E124" s="2"/>
       <c r="F124" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G124" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H124" t="s" s="2">
         <v>77</v>
@@ -15917,17 +15974,15 @@
         <v>77</v>
       </c>
       <c r="K124" t="s" s="2">
-        <v>132</v>
+        <v>447</v>
       </c>
       <c r="L124" t="s" s="2">
-        <v>178</v>
+        <v>448</v>
       </c>
       <c r="M124" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="N124" t="s" s="2">
-        <v>150</v>
-      </c>
+        <v>449</v>
+      </c>
+      <c r="N124" s="2"/>
       <c r="O124" s="2"/>
       <c r="P124" t="s" s="2">
         <v>77</v>
@@ -15994,7 +16049,7 @@
         <v>77</v>
       </c>
       <c r="AL124" t="s" s="2">
-        <v>176</v>
+        <v>77</v>
       </c>
       <c r="AM124" t="s" s="2">
         <v>77</v>
@@ -16012,39 +16067,35 @@
       </c>
       <c r="C125" s="2"/>
       <c r="D125" t="s" s="2">
-        <v>417</v>
+        <v>77</v>
       </c>
       <c r="E125" s="2"/>
       <c r="F125" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G125" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H125" t="s" s="2">
         <v>77</v>
       </c>
       <c r="I125" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="J125" t="s" s="2">
         <v>88</v>
       </c>
       <c r="K125" t="s" s="2">
-        <v>132</v>
+        <v>451</v>
       </c>
       <c r="L125" t="s" s="2">
-        <v>418</v>
+        <v>452</v>
       </c>
       <c r="M125" t="s" s="2">
-        <v>419</v>
-      </c>
-      <c r="N125" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>151</v>
-      </c>
+        <v>453</v>
+      </c>
+      <c r="N125" s="2"/>
+      <c r="O125" s="2"/>
       <c r="P125" t="s" s="2">
         <v>77</v>
       </c>
@@ -16092,25 +16143,25 @@
         <v>77</v>
       </c>
       <c r="AF125" t="s" s="2">
-        <v>420</v>
+        <v>454</v>
       </c>
       <c r="AG125" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH125" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI125" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ125" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK125" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL125" t="s" s="2">
-        <v>130</v>
+        <v>455</v>
       </c>
       <c r="AM125" t="s" s="2">
         <v>77</v>
@@ -16121,10 +16172,10 @@
     </row>
     <row r="126" hidden="true">
       <c r="A126" t="s" s="2">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="C126" s="2"/>
       <c r="D126" t="s" s="2">
@@ -16144,16 +16195,16 @@
         <v>77</v>
       </c>
       <c r="J126" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K126" t="s" s="2">
-        <v>172</v>
+        <v>451</v>
       </c>
       <c r="L126" t="s" s="2">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="M126" t="s" s="2">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="N126" s="2"/>
       <c r="O126" s="2"/>
@@ -16204,7 +16255,7 @@
         <v>77</v>
       </c>
       <c r="AF126" t="s" s="2">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="AG126" t="s" s="2">
         <v>78</v>
@@ -16219,24 +16270,24 @@
         <v>99</v>
       </c>
       <c r="AK126" t="s" s="2">
-        <v>355</v>
+        <v>77</v>
       </c>
       <c r="AL126" t="s" s="2">
-        <v>158</v>
+        <v>460</v>
       </c>
       <c r="AM126" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN126" t="s" s="2">
-        <v>454</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="127" hidden="true">
+    <row r="127">
       <c r="A127" t="s" s="2">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="C127" s="2"/>
       <c r="D127" t="s" s="2">
@@ -16250,7 +16301,7 @@
         <v>87</v>
       </c>
       <c r="H127" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I127" t="s" s="2">
         <v>77</v>
@@ -16259,13 +16310,13 @@
         <v>77</v>
       </c>
       <c r="K127" t="s" s="2">
-        <v>456</v>
+        <v>410</v>
       </c>
       <c r="L127" t="s" s="2">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="M127" t="s" s="2">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="N127" s="2"/>
       <c r="O127" s="2"/>
@@ -16316,7 +16367,7 @@
         <v>77</v>
       </c>
       <c r="AF127" t="s" s="2">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="AG127" t="s" s="2">
         <v>78</v>
@@ -16334,17 +16385,583 @@
         <v>355</v>
       </c>
       <c r="AL127" t="s" s="2">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="AM127" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN127" t="s" s="2">
-        <v>460</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="128" hidden="true">
+      <c r="A128" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="B128" t="s" s="2">
+        <v>465</v>
+      </c>
+      <c r="C128" s="2"/>
+      <c r="D128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E128" s="2"/>
+      <c r="F128" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G128" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K128" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="L128" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="M128" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="N128" s="2"/>
+      <c r="O128" s="2"/>
+      <c r="P128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q128" s="2"/>
+      <c r="R128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF128" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AG128" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH128" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AK128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL128" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="AM128" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN128" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="129" hidden="true">
+      <c r="A129" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="B129" t="s" s="2">
+        <v>466</v>
+      </c>
+      <c r="C129" s="2"/>
+      <c r="D129" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="E129" s="2"/>
+      <c r="F129" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G129" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K129" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="L129" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="M129" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="N129" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="O129" s="2"/>
+      <c r="P129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q129" s="2"/>
+      <c r="R129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF129" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="AG129" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH129" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ129" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL129" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="AM129" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN129" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="130" hidden="true">
+      <c r="A130" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="B130" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="C130" s="2"/>
+      <c r="D130" t="s" s="2">
+        <v>417</v>
+      </c>
+      <c r="E130" s="2"/>
+      <c r="F130" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G130" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I130" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="J130" t="s" s="2">
+        <v>88</v>
+      </c>
+      <c r="K130" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="L130" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="M130" t="s" s="2">
+        <v>419</v>
+      </c>
+      <c r="N130" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="O130" t="s" s="2">
+        <v>151</v>
+      </c>
+      <c r="P130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q130" s="2"/>
+      <c r="R130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF130" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AG130" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH130" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AI130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ130" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AK130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AL130" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="AM130" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN130" t="s" s="2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="131" hidden="true">
+      <c r="A131" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="B131" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="C131" s="2"/>
+      <c r="D131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E131" s="2"/>
+      <c r="F131" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G131" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K131" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="L131" t="s" s="2">
+        <v>469</v>
+      </c>
+      <c r="M131" t="s" s="2">
+        <v>470</v>
+      </c>
+      <c r="N131" s="2"/>
+      <c r="O131" s="2"/>
+      <c r="P131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q131" s="2"/>
+      <c r="R131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF131" t="s" s="2">
+        <v>468</v>
+      </c>
+      <c r="AG131" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH131" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ131" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK131" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AL131" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="AM131" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN131" t="s" s="2">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="132" hidden="true">
+      <c r="A132" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="B132" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="C132" s="2"/>
+      <c r="D132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="E132" s="2"/>
+      <c r="F132" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="G132" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="H132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="I132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="J132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="K132" t="s" s="2">
+        <v>473</v>
+      </c>
+      <c r="L132" t="s" s="2">
+        <v>474</v>
+      </c>
+      <c r="M132" t="s" s="2">
+        <v>475</v>
+      </c>
+      <c r="N132" s="2"/>
+      <c r="O132" s="2"/>
+      <c r="P132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Q132" s="2"/>
+      <c r="R132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="S132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="T132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="U132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF132" t="s" s="2">
+        <v>472</v>
+      </c>
+      <c r="AG132" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AH132" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AI132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AJ132" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AK132" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AL132" t="s" s="2">
+        <v>476</v>
+      </c>
+      <c r="AM132" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AN132" t="s" s="2">
+        <v>477</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN127">
+  <autoFilter ref="A1:AN132">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -16354,7 +16971,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI126">
+  <conditionalFormatting sqref="A2:AI131">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>